<commit_message>
Os slots de compra saem do catalogo, e nao de um 4 chutado
Defeito meu, achado rodando a conta em vez de olhar: com 4 slots por grupo a
ficha ja nao fechava no nivel 6 do Servo, e nem no 14 de uma ficha comum. Um
Servo de nivel 30 tem 54 pontos e comporta ate 9 Traco e 6 Comando, comprando
os mais baratos.

Agora a quantidade de slots e derivada -- o maior orcamento que existe contra
as entradas mais baratas do catalogo -- e da 9 e 6. O conferir-invocacao.py
recalcula esse par do json e falha se a planilha tiver outro numero, entao um
Traco novo no catalogo passa a cobrar o slot sozinho.

A regressao ganhou o caso que faltava: a montagem mais CARA que o orcamento
paga, com contra-teste provando que ela nao caberia em 4 slots.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rf8hHLmkWyinqGzFtPMHhG
</commit_message>
<xml_diff>
--- a/ficha-invocacao/ficha-invocacao.xlsx
+++ b/ficha-invocacao/ficha-invocacao.xlsx
@@ -219,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -319,6 +319,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -708,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AT96"/>
+  <dimension ref="A1:AT101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2847,7 +2853,7 @@
       <c r="C64" s="5" t="n"/>
       <c r="D64" s="26" t="inlineStr">
         <is>
-          <t>TRAÇO</t>
+          <t>TRAÇO · até 9</t>
         </is>
       </c>
       <c r="V64" s="5" t="n"/>
@@ -2856,7 +2862,7 @@
       <c r="Y64" s="5" t="n"/>
       <c r="Z64" s="26" t="inlineStr">
         <is>
-          <t>COMANDO</t>
+          <t>COMANDO · até 6</t>
         </is>
       </c>
       <c r="AR64" s="5" t="n"/>
@@ -2987,46 +2993,28 @@
       <c r="A69" s="1" t="n"/>
       <c r="B69" s="1" t="n"/>
       <c r="C69" s="5" t="n"/>
-      <c r="D69" s="5" t="n"/>
-      <c r="E69" s="5" t="n"/>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="5" t="n"/>
-      <c r="H69" s="5" t="n"/>
-      <c r="I69" s="5" t="n"/>
-      <c r="J69" s="5" t="n"/>
-      <c r="K69" s="5" t="n"/>
-      <c r="L69" s="5" t="n"/>
-      <c r="M69" s="5" t="n"/>
-      <c r="N69" s="5" t="n"/>
-      <c r="O69" s="5" t="n"/>
-      <c r="P69" s="5" t="n"/>
-      <c r="Q69" s="5" t="n"/>
-      <c r="R69" s="5" t="n"/>
-      <c r="S69" s="5" t="n"/>
-      <c r="T69" s="5" t="n"/>
-      <c r="U69" s="5" t="n"/>
+      <c r="D69" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q69" s="28">
+        <f>IFERROR(VLOOKUP($D$69,DADOS!$T$3:$U$16,2,FALSE),0)</f>
+        <v/>
+      </c>
       <c r="V69" s="5" t="n"/>
       <c r="W69" s="5" t="n"/>
       <c r="X69" s="5" t="n"/>
       <c r="Y69" s="5" t="n"/>
-      <c r="Z69" s="5" t="n"/>
-      <c r="AA69" s="5" t="n"/>
-      <c r="AB69" s="5" t="n"/>
-      <c r="AC69" s="5" t="n"/>
-      <c r="AD69" s="5" t="n"/>
-      <c r="AE69" s="5" t="n"/>
-      <c r="AF69" s="5" t="n"/>
-      <c r="AG69" s="5" t="n"/>
-      <c r="AH69" s="5" t="n"/>
-      <c r="AI69" s="5" t="n"/>
-      <c r="AJ69" s="5" t="n"/>
-      <c r="AK69" s="5" t="n"/>
-      <c r="AL69" s="5" t="n"/>
-      <c r="AM69" s="5" t="n"/>
-      <c r="AN69" s="5" t="n"/>
-      <c r="AO69" s="5" t="n"/>
-      <c r="AP69" s="5" t="n"/>
-      <c r="AQ69" s="5" t="n"/>
+      <c r="Z69" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AM69" s="28">
+        <f>IFERROR(VLOOKUP($Z$69,DADOS!$W$3:$X$10,2,FALSE),0)</f>
+        <v/>
+      </c>
       <c r="AR69" s="5" t="n"/>
       <c r="AS69" s="5" t="n"/>
       <c r="AT69" s="5" t="n"/>
@@ -3035,87 +3023,123 @@
       <c r="A70" s="1" t="n"/>
       <c r="B70" s="1" t="n"/>
       <c r="C70" s="5" t="n"/>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>GASTO</t>
-        </is>
-      </c>
-      <c r="K70" s="5" t="n"/>
-      <c r="L70" s="8" t="inlineStr">
-        <is>
-          <t>SOBRA</t>
-        </is>
-      </c>
-      <c r="S70" s="5" t="n"/>
-      <c r="T70" s="8" t="inlineStr">
-        <is>
-          <t>O QUE ELE NÃO COMPRA A PREÇO NENHUM</t>
-        </is>
-      </c>
+      <c r="D70" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q70" s="30">
+        <f>IFERROR(VLOOKUP($D$70,DADOS!$T$3:$U$16,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="V70" s="5" t="n"/>
+      <c r="W70" s="5" t="n"/>
+      <c r="X70" s="5" t="n"/>
+      <c r="Y70" s="5" t="n"/>
+      <c r="Z70" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AM70" s="30">
+        <f>IFERROR(VLOOKUP($Z$70,DADOS!$W$3:$X$10,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="AR70" s="5" t="n"/>
+      <c r="AS70" s="5" t="n"/>
+      <c r="AT70" s="5" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="1" t="n"/>
       <c r="B71" s="1" t="n"/>
       <c r="C71" s="5" t="n"/>
-      <c r="D71" s="24">
-        <f>$Q$65+$Q$66+$Q$67+$Q$68+$AM$65+$AM$66+$AM$67+$AM$68</f>
+      <c r="D71" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q71" s="28">
+        <f>IFERROR(VLOOKUP($D$71,DADOS!$T$3:$U$16,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="K71" s="5" t="n"/>
-      <c r="L71" s="31">
-        <f>IF($D$61-($Q$65+$Q$66+$Q$67+$Q$68+$AM$65+$AM$66+$AM$67+$AM$68)&lt;0,"estourou "&amp;(($Q$65+$Q$66+$Q$67+$Q$68+$AM$65+$AM$66+$AM$67+$AM$68)-$D$61),$D$61-($Q$65+$Q$66+$Q$67+$Q$68+$AM$65+$AM$66+$AM$67+$AM$68))</f>
-        <v/>
-      </c>
-      <c r="S71" s="5" t="n"/>
-      <c r="T71" s="25" t="inlineStr">
-        <is>
-          <t>dado de dano · qualquer coisa que cresça com refino · atributo · Defesa, acerto ou vida direto</t>
-        </is>
-      </c>
+      <c r="V71" s="5" t="n"/>
+      <c r="W71" s="5" t="n"/>
+      <c r="X71" s="5" t="n"/>
+      <c r="Y71" s="5" t="n"/>
+      <c r="Z71" s="5" t="n"/>
+      <c r="AA71" s="5" t="n"/>
+      <c r="AB71" s="5" t="n"/>
+      <c r="AC71" s="5" t="n"/>
+      <c r="AD71" s="5" t="n"/>
+      <c r="AE71" s="5" t="n"/>
+      <c r="AF71" s="5" t="n"/>
+      <c r="AG71" s="5" t="n"/>
+      <c r="AH71" s="5" t="n"/>
+      <c r="AI71" s="5" t="n"/>
+      <c r="AJ71" s="5" t="n"/>
+      <c r="AK71" s="5" t="n"/>
+      <c r="AL71" s="5" t="n"/>
+      <c r="AM71" s="5" t="n"/>
+      <c r="AN71" s="5" t="n"/>
+      <c r="AO71" s="5" t="n"/>
+      <c r="AP71" s="5" t="n"/>
+      <c r="AQ71" s="5" t="n"/>
+      <c r="AR71" s="5" t="n"/>
+      <c r="AS71" s="5" t="n"/>
+      <c r="AT71" s="5" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="1" t="n"/>
       <c r="B72" s="1" t="n"/>
       <c r="C72" s="5" t="n"/>
-      <c r="D72" s="13" t="n"/>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="n"/>
-      <c r="I72" s="13" t="n"/>
-      <c r="J72" s="13" t="n"/>
-      <c r="K72" s="5" t="n"/>
-      <c r="L72" s="13" t="n"/>
-      <c r="M72" s="13" t="n"/>
-      <c r="N72" s="13" t="n"/>
-      <c r="O72" s="13" t="n"/>
-      <c r="P72" s="13" t="n"/>
-      <c r="Q72" s="13" t="n"/>
-      <c r="R72" s="13" t="n"/>
-      <c r="S72" s="5" t="n"/>
+      <c r="D72" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q72" s="30">
+        <f>IFERROR(VLOOKUP($D$72,DADOS!$T$3:$U$16,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="V72" s="5" t="n"/>
+      <c r="W72" s="5" t="n"/>
+      <c r="X72" s="5" t="n"/>
+      <c r="Y72" s="5" t="n"/>
+      <c r="Z72" s="5" t="n"/>
+      <c r="AA72" s="5" t="n"/>
+      <c r="AB72" s="5" t="n"/>
+      <c r="AC72" s="5" t="n"/>
+      <c r="AD72" s="5" t="n"/>
+      <c r="AE72" s="5" t="n"/>
+      <c r="AF72" s="5" t="n"/>
+      <c r="AG72" s="5" t="n"/>
+      <c r="AH72" s="5" t="n"/>
+      <c r="AI72" s="5" t="n"/>
+      <c r="AJ72" s="5" t="n"/>
+      <c r="AK72" s="5" t="n"/>
+      <c r="AL72" s="5" t="n"/>
+      <c r="AM72" s="5" t="n"/>
+      <c r="AN72" s="5" t="n"/>
+      <c r="AO72" s="5" t="n"/>
+      <c r="AP72" s="5" t="n"/>
+      <c r="AQ72" s="5" t="n"/>
+      <c r="AR72" s="5" t="n"/>
+      <c r="AS72" s="5" t="n"/>
+      <c r="AT72" s="5" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="1" t="n"/>
       <c r="B73" s="1" t="n"/>
       <c r="C73" s="5" t="n"/>
-      <c r="D73" s="5" t="n"/>
-      <c r="E73" s="5" t="n"/>
-      <c r="F73" s="5" t="n"/>
-      <c r="G73" s="5" t="n"/>
-      <c r="H73" s="5" t="n"/>
-      <c r="I73" s="5" t="n"/>
-      <c r="J73" s="5" t="n"/>
-      <c r="K73" s="5" t="n"/>
-      <c r="L73" s="5" t="n"/>
-      <c r="M73" s="5" t="n"/>
-      <c r="N73" s="5" t="n"/>
-      <c r="O73" s="5" t="n"/>
-      <c r="P73" s="5" t="n"/>
-      <c r="Q73" s="5" t="n"/>
-      <c r="R73" s="5" t="n"/>
-      <c r="S73" s="5" t="n"/>
-      <c r="T73" s="5" t="n"/>
-      <c r="U73" s="5" t="n"/>
+      <c r="D73" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q73" s="28">
+        <f>IFERROR(VLOOKUP($D$73,DADOS!$T$3:$U$16,2,FALSE),0)</f>
+        <v/>
+      </c>
       <c r="V73" s="5" t="n"/>
       <c r="W73" s="5" t="n"/>
       <c r="X73" s="5" t="n"/>
@@ -3146,150 +3170,138 @@
       <c r="A74" s="1" t="n"/>
       <c r="B74" s="1" t="n"/>
       <c r="C74" s="5" t="n"/>
-      <c r="D74" s="14" t="inlineStr">
-        <is>
-          <t>o Servo monta com o orçamento da ficha mais metade, porque é um corpo só e não cinco. Todo orçamento é múltiplo de 4, então fecha redondo.</t>
-        </is>
-      </c>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="5" t="n"/>
+      <c r="J74" s="5" t="n"/>
+      <c r="K74" s="5" t="n"/>
+      <c r="L74" s="5" t="n"/>
+      <c r="M74" s="5" t="n"/>
+      <c r="N74" s="5" t="n"/>
+      <c r="O74" s="5" t="n"/>
+      <c r="P74" s="5" t="n"/>
+      <c r="Q74" s="5" t="n"/>
+      <c r="R74" s="5" t="n"/>
+      <c r="S74" s="5" t="n"/>
+      <c r="T74" s="5" t="n"/>
+      <c r="U74" s="5" t="n"/>
+      <c r="V74" s="5" t="n"/>
+      <c r="W74" s="5" t="n"/>
+      <c r="X74" s="5" t="n"/>
+      <c r="Y74" s="5" t="n"/>
+      <c r="Z74" s="5" t="n"/>
+      <c r="AA74" s="5" t="n"/>
+      <c r="AB74" s="5" t="n"/>
+      <c r="AC74" s="5" t="n"/>
+      <c r="AD74" s="5" t="n"/>
+      <c r="AE74" s="5" t="n"/>
+      <c r="AF74" s="5" t="n"/>
+      <c r="AG74" s="5" t="n"/>
+      <c r="AH74" s="5" t="n"/>
+      <c r="AI74" s="5" t="n"/>
+      <c r="AJ74" s="5" t="n"/>
+      <c r="AK74" s="5" t="n"/>
+      <c r="AL74" s="5" t="n"/>
+      <c r="AM74" s="5" t="n"/>
+      <c r="AN74" s="5" t="n"/>
+      <c r="AO74" s="5" t="n"/>
+      <c r="AP74" s="5" t="n"/>
+      <c r="AQ74" s="5" t="n"/>
+      <c r="AR74" s="5" t="n"/>
+      <c r="AS74" s="5" t="n"/>
+      <c r="AT74" s="5" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="1" t="n"/>
       <c r="B75" s="1" t="n"/>
       <c r="C75" s="5" t="n"/>
-      <c r="D75" s="5" t="n"/>
-      <c r="E75" s="5" t="n"/>
-      <c r="F75" s="5" t="n"/>
-      <c r="G75" s="5" t="n"/>
-      <c r="H75" s="5" t="n"/>
-      <c r="I75" s="5" t="n"/>
-      <c r="J75" s="5" t="n"/>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>GASTO</t>
+        </is>
+      </c>
       <c r="K75" s="5" t="n"/>
-      <c r="L75" s="5" t="n"/>
-      <c r="M75" s="5" t="n"/>
-      <c r="N75" s="5" t="n"/>
-      <c r="O75" s="5" t="n"/>
-      <c r="P75" s="5" t="n"/>
-      <c r="Q75" s="5" t="n"/>
-      <c r="R75" s="5" t="n"/>
+      <c r="L75" s="8" t="inlineStr">
+        <is>
+          <t>SOBRA</t>
+        </is>
+      </c>
       <c r="S75" s="5" t="n"/>
-      <c r="T75" s="5" t="n"/>
-      <c r="U75" s="5" t="n"/>
-      <c r="V75" s="5" t="n"/>
-      <c r="W75" s="5" t="n"/>
-      <c r="X75" s="5" t="n"/>
-      <c r="Y75" s="5" t="n"/>
-      <c r="Z75" s="5" t="n"/>
-      <c r="AA75" s="5" t="n"/>
-      <c r="AB75" s="5" t="n"/>
-      <c r="AC75" s="5" t="n"/>
-      <c r="AD75" s="5" t="n"/>
-      <c r="AE75" s="5" t="n"/>
-      <c r="AF75" s="5" t="n"/>
-      <c r="AG75" s="5" t="n"/>
-      <c r="AH75" s="5" t="n"/>
-      <c r="AI75" s="5" t="n"/>
-      <c r="AJ75" s="5" t="n"/>
-      <c r="AK75" s="5" t="n"/>
-      <c r="AL75" s="5" t="n"/>
-      <c r="AM75" s="5" t="n"/>
-      <c r="AN75" s="5" t="n"/>
-      <c r="AO75" s="5" t="n"/>
-      <c r="AP75" s="5" t="n"/>
-      <c r="AQ75" s="5" t="n"/>
-      <c r="AR75" s="5" t="n"/>
-      <c r="AS75" s="5" t="n"/>
-      <c r="AT75" s="5" t="n"/>
+      <c r="T75" s="8" t="inlineStr">
+        <is>
+          <t>O QUE ELE NÃO COMPRA A PREÇO NENHUM</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="1" t="n"/>
       <c r="B76" s="1" t="n"/>
       <c r="C76" s="5" t="n"/>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
-        <is>
-          <t>INVESTIR — o ataque, e toda invocação tem</t>
-        </is>
-      </c>
-      <c r="AG76" s="5" t="n"/>
-      <c r="AH76" s="5" t="n"/>
-      <c r="AI76" s="5" t="n"/>
-      <c r="AJ76" s="5" t="n"/>
-      <c r="AK76" s="5" t="n"/>
-      <c r="AL76" s="5" t="n"/>
-      <c r="AM76" s="5" t="n"/>
-      <c r="AN76" s="5" t="n"/>
-      <c r="AO76" s="5" t="n"/>
-      <c r="AP76" s="5" t="n"/>
-      <c r="AQ76" s="5" t="n"/>
-      <c r="AR76" s="5" t="n"/>
-      <c r="AS76" s="5" t="n"/>
-      <c r="AT76" s="5" t="n"/>
+      <c r="D76" s="24">
+        <f>$Q$65+$Q$66+$Q$67+$Q$68+$Q$69+$Q$70+$Q$71+$Q$72+$Q$73+$AM$65+$AM$66+$AM$67+$AM$68+$AM$69+$AM$70</f>
+        <v/>
+      </c>
+      <c r="K76" s="5" t="n"/>
+      <c r="L76" s="31">
+        <f>IF($D$61-($Q$65+$Q$66+$Q$67+$Q$68+$Q$69+$Q$70+$Q$71+$Q$72+$Q$73+$AM$65+$AM$66+$AM$67+$AM$68+$AM$69+$AM$70)&lt;0,"estourou "&amp;(($Q$65+$Q$66+$Q$67+$Q$68+$Q$69+$Q$70+$Q$71+$Q$72+$Q$73+$AM$65+$AM$66+$AM$67+$AM$68+$AM$69+$AM$70)-$D$61),$D$61-($Q$65+$Q$66+$Q$67+$Q$68+$Q$69+$Q$70+$Q$71+$Q$72+$Q$73+$AM$65+$AM$66+$AM$67+$AM$68+$AM$69+$AM$70))</f>
+        <v/>
+      </c>
+      <c r="S76" s="5" t="n"/>
+      <c r="T76" s="25" t="inlineStr">
+        <is>
+          <t>dado de dano · qualquer coisa que cresça com refino · atributo · Defesa, acerto ou vida direto</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="1" t="n"/>
       <c r="B77" s="1" t="n"/>
       <c r="C77" s="5" t="n"/>
-      <c r="G77" s="5" t="n"/>
-      <c r="H77" s="5" t="n"/>
-      <c r="I77" s="5" t="n"/>
-      <c r="J77" s="5" t="n"/>
+      <c r="D77" s="13" t="n"/>
+      <c r="E77" s="13" t="n"/>
+      <c r="F77" s="13" t="n"/>
+      <c r="G77" s="13" t="n"/>
+      <c r="H77" s="13" t="n"/>
+      <c r="I77" s="13" t="n"/>
+      <c r="J77" s="13" t="n"/>
       <c r="K77" s="5" t="n"/>
-      <c r="L77" s="5" t="n"/>
-      <c r="M77" s="5" t="n"/>
-      <c r="N77" s="5" t="n"/>
-      <c r="O77" s="5" t="n"/>
-      <c r="P77" s="5" t="n"/>
-      <c r="Q77" s="5" t="n"/>
-      <c r="R77" s="5" t="n"/>
+      <c r="L77" s="13" t="n"/>
+      <c r="M77" s="13" t="n"/>
+      <c r="N77" s="13" t="n"/>
+      <c r="O77" s="13" t="n"/>
+      <c r="P77" s="13" t="n"/>
+      <c r="Q77" s="13" t="n"/>
+      <c r="R77" s="13" t="n"/>
       <c r="S77" s="5" t="n"/>
-      <c r="T77" s="5" t="n"/>
-      <c r="U77" s="5" t="n"/>
-      <c r="V77" s="5" t="n"/>
-      <c r="W77" s="5" t="n"/>
-      <c r="X77" s="5" t="n"/>
-      <c r="Y77" s="5" t="n"/>
-      <c r="Z77" s="5" t="n"/>
-      <c r="AA77" s="5" t="n"/>
-      <c r="AB77" s="5" t="n"/>
-      <c r="AC77" s="5" t="n"/>
-      <c r="AD77" s="5" t="n"/>
-      <c r="AE77" s="5" t="n"/>
-      <c r="AF77" s="5" t="n"/>
-      <c r="AG77" s="5" t="n"/>
-      <c r="AH77" s="5" t="n"/>
-      <c r="AI77" s="5" t="n"/>
-      <c r="AJ77" s="5" t="n"/>
-      <c r="AK77" s="5" t="n"/>
-      <c r="AL77" s="5" t="n"/>
-      <c r="AM77" s="5" t="n"/>
-      <c r="AN77" s="5" t="n"/>
-      <c r="AO77" s="5" t="n"/>
-      <c r="AP77" s="5" t="n"/>
-      <c r="AQ77" s="5" t="n"/>
-      <c r="AR77" s="5" t="n"/>
-      <c r="AS77" s="5" t="n"/>
-      <c r="AT77" s="5" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="1" t="n"/>
       <c r="B78" s="1" t="n"/>
       <c r="C78" s="5" t="n"/>
-      <c r="D78" s="8" t="inlineStr">
-        <is>
-          <t>DANO DO INVESTIR</t>
-        </is>
-      </c>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="5" t="n"/>
+      <c r="I78" s="5" t="n"/>
+      <c r="J78" s="5" t="n"/>
+      <c r="K78" s="5" t="n"/>
       <c r="L78" s="5" t="n"/>
       <c r="M78" s="5" t="n"/>
-      <c r="N78" s="8" t="inlineStr">
-        <is>
-          <t>POR CORPO</t>
-        </is>
-      </c>
+      <c r="N78" s="5" t="n"/>
+      <c r="O78" s="5" t="n"/>
+      <c r="P78" s="5" t="n"/>
+      <c r="Q78" s="5" t="n"/>
+      <c r="R78" s="5" t="n"/>
+      <c r="S78" s="5" t="n"/>
+      <c r="T78" s="5" t="n"/>
+      <c r="U78" s="5" t="n"/>
+      <c r="V78" s="5" t="n"/>
+      <c r="W78" s="5" t="n"/>
+      <c r="X78" s="5" t="n"/>
       <c r="Y78" s="5" t="n"/>
       <c r="Z78" s="5" t="n"/>
       <c r="AA78" s="5" t="n"/>
@@ -3317,45 +3329,24 @@
       <c r="A79" s="1" t="n"/>
       <c r="B79" s="1" t="n"/>
       <c r="C79" s="5" t="n"/>
-      <c r="D79" s="22">
-        <f>IF($D$7="","",VLOOKUP($D$7,DADOS!$Z$3:$AB$9,IF($AA$14="Matilha",3,2),TRUE))</f>
-        <v/>
-      </c>
-      <c r="L79" s="5" t="n"/>
-      <c r="M79" s="5" t="n"/>
-      <c r="N79" s="32">
-        <f>IF($AA$14="Matilha","cada um dos cinco rola isto",IF($AA$14="","","o corpo em campo rola isto"))</f>
-        <v/>
-      </c>
-      <c r="AE79" s="5" t="n"/>
-      <c r="AF79" s="5" t="n"/>
-      <c r="AG79" s="5" t="n"/>
-      <c r="AH79" s="5" t="n"/>
-      <c r="AI79" s="5" t="n"/>
-      <c r="AJ79" s="5" t="n"/>
-      <c r="AK79" s="5" t="n"/>
-      <c r="AL79" s="5" t="n"/>
-      <c r="AM79" s="5" t="n"/>
-      <c r="AN79" s="5" t="n"/>
-      <c r="AO79" s="5" t="n"/>
-      <c r="AP79" s="5" t="n"/>
-      <c r="AQ79" s="5" t="n"/>
-      <c r="AR79" s="5" t="n"/>
-      <c r="AS79" s="5" t="n"/>
-      <c r="AT79" s="5" t="n"/>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>o Servo monta com o orçamento da ficha mais metade, porque é um corpo só e não cinco. Todo orçamento é múltiplo de 4, então fecha redondo.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="1" t="n"/>
       <c r="B80" s="1" t="n"/>
       <c r="C80" s="5" t="n"/>
-      <c r="D80" s="13" t="n"/>
-      <c r="E80" s="13" t="n"/>
-      <c r="F80" s="13" t="n"/>
-      <c r="G80" s="13" t="n"/>
-      <c r="H80" s="13" t="n"/>
-      <c r="I80" s="13" t="n"/>
-      <c r="J80" s="13" t="n"/>
-      <c r="K80" s="13" t="n"/>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="5" t="n"/>
+      <c r="F80" s="5" t="n"/>
+      <c r="G80" s="5" t="n"/>
+      <c r="H80" s="5" t="n"/>
+      <c r="I80" s="5" t="n"/>
+      <c r="J80" s="5" t="n"/>
+      <c r="K80" s="5" t="n"/>
       <c r="L80" s="5" t="n"/>
       <c r="M80" s="5" t="n"/>
       <c r="N80" s="5" t="n"/>
@@ -3396,19 +3387,35 @@
       <c r="A81" s="1" t="n"/>
       <c r="B81" s="1" t="n"/>
       <c r="C81" s="5" t="n"/>
-      <c r="D81" s="14" t="inlineStr">
-        <is>
-          <t>você e todas as suas invocações somados entregam uma Rotina. O número de dados sempre desce — a soma nunca passa do que você faria sozinho.</t>
-        </is>
-      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>INVESTIR — o ataque, e toda invocação tem</t>
+        </is>
+      </c>
+      <c r="AG81" s="5" t="n"/>
+      <c r="AH81" s="5" t="n"/>
+      <c r="AI81" s="5" t="n"/>
+      <c r="AJ81" s="5" t="n"/>
+      <c r="AK81" s="5" t="n"/>
+      <c r="AL81" s="5" t="n"/>
+      <c r="AM81" s="5" t="n"/>
+      <c r="AN81" s="5" t="n"/>
+      <c r="AO81" s="5" t="n"/>
+      <c r="AP81" s="5" t="n"/>
+      <c r="AQ81" s="5" t="n"/>
+      <c r="AR81" s="5" t="n"/>
+      <c r="AS81" s="5" t="n"/>
+      <c r="AT81" s="5" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="1" t="n"/>
       <c r="B82" s="1" t="n"/>
       <c r="C82" s="5" t="n"/>
-      <c r="D82" s="5" t="n"/>
-      <c r="E82" s="5" t="n"/>
-      <c r="F82" s="5" t="n"/>
       <c r="G82" s="5" t="n"/>
       <c r="H82" s="5" t="n"/>
       <c r="I82" s="5" t="n"/>
@@ -3454,16 +3461,24 @@
       <c r="A83" s="1" t="n"/>
       <c r="B83" s="1" t="n"/>
       <c r="C83" s="5" t="n"/>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="inlineStr">
-        <is>
-          <t>NA MESA — o que não muda</t>
-        </is>
-      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>DANO DO INVESTIR</t>
+        </is>
+      </c>
+      <c r="L83" s="5" t="n"/>
+      <c r="M83" s="5" t="n"/>
+      <c r="N83" s="8" t="inlineStr">
+        <is>
+          <t>POR CORPO</t>
+        </is>
+      </c>
+      <c r="Y83" s="5" t="n"/>
+      <c r="Z83" s="5" t="n"/>
+      <c r="AA83" s="5" t="n"/>
+      <c r="AB83" s="5" t="n"/>
+      <c r="AC83" s="5" t="n"/>
+      <c r="AD83" s="5" t="n"/>
       <c r="AE83" s="5" t="n"/>
       <c r="AF83" s="5" t="n"/>
       <c r="AG83" s="5" t="n"/>
@@ -3485,30 +3500,16 @@
       <c r="A84" s="1" t="n"/>
       <c r="B84" s="1" t="n"/>
       <c r="C84" s="5" t="n"/>
-      <c r="G84" s="5" t="n"/>
-      <c r="H84" s="5" t="n"/>
-      <c r="I84" s="5" t="n"/>
-      <c r="J84" s="5" t="n"/>
-      <c r="K84" s="5" t="n"/>
+      <c r="D84" s="22">
+        <f>IF($D$7="","",VLOOKUP($D$7,DADOS!$Z$3:$AB$9,IF($AA$14="Matilha",3,2),TRUE))</f>
+        <v/>
+      </c>
       <c r="L84" s="5" t="n"/>
       <c r="M84" s="5" t="n"/>
-      <c r="N84" s="5" t="n"/>
-      <c r="O84" s="5" t="n"/>
-      <c r="P84" s="5" t="n"/>
-      <c r="Q84" s="5" t="n"/>
-      <c r="R84" s="5" t="n"/>
-      <c r="S84" s="5" t="n"/>
-      <c r="T84" s="5" t="n"/>
-      <c r="U84" s="5" t="n"/>
-      <c r="V84" s="5" t="n"/>
-      <c r="W84" s="5" t="n"/>
-      <c r="X84" s="5" t="n"/>
-      <c r="Y84" s="5" t="n"/>
-      <c r="Z84" s="5" t="n"/>
-      <c r="AA84" s="5" t="n"/>
-      <c r="AB84" s="5" t="n"/>
-      <c r="AC84" s="5" t="n"/>
-      <c r="AD84" s="5" t="n"/>
+      <c r="N84" s="32">
+        <f>IF($AA$14="Matilha","cada um dos cinco rola isto",IF($AA$14="","","o corpo em campo rola isto"))</f>
+        <v/>
+      </c>
       <c r="AE84" s="5" t="n"/>
       <c r="AF84" s="5" t="n"/>
       <c r="AG84" s="5" t="n"/>
@@ -3530,246 +3531,315 @@
       <c r="A85" s="1" t="n"/>
       <c r="B85" s="1" t="n"/>
       <c r="C85" s="5" t="n"/>
-      <c r="D85" s="33" t="inlineStr">
-        <is>
-          <t>invocar</t>
-        </is>
-      </c>
-      <c r="M85" s="34">
-        <f>("custa "&amp;$AM$7&amp;" PE e a Ação Padrão")</f>
-        <v/>
-      </c>
+      <c r="D85" s="13" t="n"/>
+      <c r="E85" s="13" t="n"/>
+      <c r="F85" s="13" t="n"/>
+      <c r="G85" s="13" t="n"/>
+      <c r="H85" s="13" t="n"/>
+      <c r="I85" s="13" t="n"/>
+      <c r="J85" s="13" t="n"/>
+      <c r="K85" s="13" t="n"/>
+      <c r="L85" s="5" t="n"/>
+      <c r="M85" s="5" t="n"/>
+      <c r="N85" s="5" t="n"/>
+      <c r="O85" s="5" t="n"/>
+      <c r="P85" s="5" t="n"/>
+      <c r="Q85" s="5" t="n"/>
+      <c r="R85" s="5" t="n"/>
+      <c r="S85" s="5" t="n"/>
+      <c r="T85" s="5" t="n"/>
+      <c r="U85" s="5" t="n"/>
+      <c r="V85" s="5" t="n"/>
+      <c r="W85" s="5" t="n"/>
+      <c r="X85" s="5" t="n"/>
+      <c r="Y85" s="5" t="n"/>
+      <c r="Z85" s="5" t="n"/>
+      <c r="AA85" s="5" t="n"/>
+      <c r="AB85" s="5" t="n"/>
+      <c r="AC85" s="5" t="n"/>
+      <c r="AD85" s="5" t="n"/>
+      <c r="AE85" s="5" t="n"/>
+      <c r="AF85" s="5" t="n"/>
+      <c r="AG85" s="5" t="n"/>
+      <c r="AH85" s="5" t="n"/>
+      <c r="AI85" s="5" t="n"/>
+      <c r="AJ85" s="5" t="n"/>
+      <c r="AK85" s="5" t="n"/>
+      <c r="AL85" s="5" t="n"/>
+      <c r="AM85" s="5" t="n"/>
+      <c r="AN85" s="5" t="n"/>
+      <c r="AO85" s="5" t="n"/>
+      <c r="AP85" s="5" t="n"/>
+      <c r="AQ85" s="5" t="n"/>
+      <c r="AR85" s="5" t="n"/>
+      <c r="AS85" s="5" t="n"/>
+      <c r="AT85" s="5" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="1" t="n"/>
       <c r="B86" s="1" t="n"/>
       <c r="C86" s="5" t="n"/>
-      <c r="D86" s="35" t="inlineStr">
-        <is>
-          <t>comandar</t>
-        </is>
-      </c>
-      <c r="M86" s="36">
-        <f>"a Ação Padrão, toda rodada"</f>
-        <v/>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>você e todas as suas invocações somados entregam uma Rotina. O número de dados sempre desce — a soma nunca passa do que você faria sozinho.</t>
+        </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="1" t="n"/>
       <c r="B87" s="1" t="n"/>
       <c r="C87" s="5" t="n"/>
-      <c r="D87" s="33" t="inlineStr">
-        <is>
-          <t>iniciativa</t>
-        </is>
-      </c>
-      <c r="M87" s="34">
-        <f>"a sua, e ela age logo depois de você"</f>
-        <v/>
-      </c>
+      <c r="D87" s="5" t="n"/>
+      <c r="E87" s="5" t="n"/>
+      <c r="F87" s="5" t="n"/>
+      <c r="G87" s="5" t="n"/>
+      <c r="H87" s="5" t="n"/>
+      <c r="I87" s="5" t="n"/>
+      <c r="J87" s="5" t="n"/>
+      <c r="K87" s="5" t="n"/>
+      <c r="L87" s="5" t="n"/>
+      <c r="M87" s="5" t="n"/>
+      <c r="N87" s="5" t="n"/>
+      <c r="O87" s="5" t="n"/>
+      <c r="P87" s="5" t="n"/>
+      <c r="Q87" s="5" t="n"/>
+      <c r="R87" s="5" t="n"/>
+      <c r="S87" s="5" t="n"/>
+      <c r="T87" s="5" t="n"/>
+      <c r="U87" s="5" t="n"/>
+      <c r="V87" s="5" t="n"/>
+      <c r="W87" s="5" t="n"/>
+      <c r="X87" s="5" t="n"/>
+      <c r="Y87" s="5" t="n"/>
+      <c r="Z87" s="5" t="n"/>
+      <c r="AA87" s="5" t="n"/>
+      <c r="AB87" s="5" t="n"/>
+      <c r="AC87" s="5" t="n"/>
+      <c r="AD87" s="5" t="n"/>
+      <c r="AE87" s="5" t="n"/>
+      <c r="AF87" s="5" t="n"/>
+      <c r="AG87" s="5" t="n"/>
+      <c r="AH87" s="5" t="n"/>
+      <c r="AI87" s="5" t="n"/>
+      <c r="AJ87" s="5" t="n"/>
+      <c r="AK87" s="5" t="n"/>
+      <c r="AL87" s="5" t="n"/>
+      <c r="AM87" s="5" t="n"/>
+      <c r="AN87" s="5" t="n"/>
+      <c r="AO87" s="5" t="n"/>
+      <c r="AP87" s="5" t="n"/>
+      <c r="AQ87" s="5" t="n"/>
+      <c r="AR87" s="5" t="n"/>
+      <c r="AS87" s="5" t="n"/>
+      <c r="AT87" s="5" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="1" t="n"/>
       <c r="B88" s="1" t="n"/>
       <c r="C88" s="5" t="n"/>
-      <c r="D88" s="35" t="inlineStr">
-        <is>
-          <t>deslocamento</t>
-        </is>
-      </c>
-      <c r="M88" s="36">
-        <f>(9&amp;" metros")</f>
-        <v/>
-      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>NA MESA — o que não muda</t>
+        </is>
+      </c>
+      <c r="AE88" s="5" t="n"/>
+      <c r="AF88" s="5" t="n"/>
+      <c r="AG88" s="5" t="n"/>
+      <c r="AH88" s="5" t="n"/>
+      <c r="AI88" s="5" t="n"/>
+      <c r="AJ88" s="5" t="n"/>
+      <c r="AK88" s="5" t="n"/>
+      <c r="AL88" s="5" t="n"/>
+      <c r="AM88" s="5" t="n"/>
+      <c r="AN88" s="5" t="n"/>
+      <c r="AO88" s="5" t="n"/>
+      <c r="AP88" s="5" t="n"/>
+      <c r="AQ88" s="5" t="n"/>
+      <c r="AR88" s="5" t="n"/>
+      <c r="AS88" s="5" t="n"/>
+      <c r="AT88" s="5" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="1" t="n"/>
       <c r="B89" s="1" t="n"/>
       <c r="C89" s="5" t="n"/>
-      <c r="D89" s="33" t="inlineStr">
-        <is>
-          <t>amarra</t>
-        </is>
-      </c>
-      <c r="M89" s="34">
-        <f>(18&amp;" metros — além disso não pode ser comandada, e não some")</f>
-        <v/>
-      </c>
+      <c r="G89" s="5" t="n"/>
+      <c r="H89" s="5" t="n"/>
+      <c r="I89" s="5" t="n"/>
+      <c r="J89" s="5" t="n"/>
+      <c r="K89" s="5" t="n"/>
+      <c r="L89" s="5" t="n"/>
+      <c r="M89" s="5" t="n"/>
+      <c r="N89" s="5" t="n"/>
+      <c r="O89" s="5" t="n"/>
+      <c r="P89" s="5" t="n"/>
+      <c r="Q89" s="5" t="n"/>
+      <c r="R89" s="5" t="n"/>
+      <c r="S89" s="5" t="n"/>
+      <c r="T89" s="5" t="n"/>
+      <c r="U89" s="5" t="n"/>
+      <c r="V89" s="5" t="n"/>
+      <c r="W89" s="5" t="n"/>
+      <c r="X89" s="5" t="n"/>
+      <c r="Y89" s="5" t="n"/>
+      <c r="Z89" s="5" t="n"/>
+      <c r="AA89" s="5" t="n"/>
+      <c r="AB89" s="5" t="n"/>
+      <c r="AC89" s="5" t="n"/>
+      <c r="AD89" s="5" t="n"/>
+      <c r="AE89" s="5" t="n"/>
+      <c r="AF89" s="5" t="n"/>
+      <c r="AG89" s="5" t="n"/>
+      <c r="AH89" s="5" t="n"/>
+      <c r="AI89" s="5" t="n"/>
+      <c r="AJ89" s="5" t="n"/>
+      <c r="AK89" s="5" t="n"/>
+      <c r="AL89" s="5" t="n"/>
+      <c r="AM89" s="5" t="n"/>
+      <c r="AN89" s="5" t="n"/>
+      <c r="AO89" s="5" t="n"/>
+      <c r="AP89" s="5" t="n"/>
+      <c r="AQ89" s="5" t="n"/>
+      <c r="AR89" s="5" t="n"/>
+      <c r="AS89" s="5" t="n"/>
+      <c r="AT89" s="5" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="1" t="n"/>
       <c r="B90" s="1" t="n"/>
       <c r="C90" s="5" t="n"/>
-      <c r="D90" s="5" t="n"/>
-      <c r="E90" s="5" t="n"/>
-      <c r="F90" s="5" t="n"/>
-      <c r="G90" s="5" t="n"/>
-      <c r="H90" s="5" t="n"/>
-      <c r="I90" s="5" t="n"/>
-      <c r="J90" s="5" t="n"/>
-      <c r="K90" s="5" t="n"/>
-      <c r="L90" s="5" t="n"/>
-      <c r="M90" s="5" t="n"/>
-      <c r="N90" s="5" t="n"/>
-      <c r="O90" s="5" t="n"/>
-      <c r="P90" s="5" t="n"/>
-      <c r="Q90" s="5" t="n"/>
-      <c r="R90" s="5" t="n"/>
-      <c r="S90" s="5" t="n"/>
-      <c r="T90" s="5" t="n"/>
-      <c r="U90" s="5" t="n"/>
-      <c r="V90" s="5" t="n"/>
-      <c r="W90" s="5" t="n"/>
-      <c r="X90" s="5" t="n"/>
-      <c r="Y90" s="5" t="n"/>
-      <c r="Z90" s="5" t="n"/>
-      <c r="AA90" s="5" t="n"/>
-      <c r="AB90" s="5" t="n"/>
-      <c r="AC90" s="5" t="n"/>
-      <c r="AD90" s="5" t="n"/>
-      <c r="AE90" s="5" t="n"/>
-      <c r="AF90" s="5" t="n"/>
-      <c r="AG90" s="5" t="n"/>
-      <c r="AH90" s="5" t="n"/>
-      <c r="AI90" s="5" t="n"/>
-      <c r="AJ90" s="5" t="n"/>
-      <c r="AK90" s="5" t="n"/>
-      <c r="AL90" s="5" t="n"/>
-      <c r="AM90" s="5" t="n"/>
-      <c r="AN90" s="5" t="n"/>
-      <c r="AO90" s="5" t="n"/>
-      <c r="AP90" s="5" t="n"/>
-      <c r="AQ90" s="5" t="n"/>
-      <c r="AR90" s="5" t="n"/>
-      <c r="AS90" s="5" t="n"/>
-      <c r="AT90" s="5" t="n"/>
+      <c r="D90" s="33" t="inlineStr">
+        <is>
+          <t>invocar</t>
+        </is>
+      </c>
+      <c r="M90" s="34">
+        <f>("custa "&amp;$AM$7&amp;" PE e a Ação Padrão")</f>
+        <v/>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="1" t="n"/>
       <c r="B91" s="1" t="n"/>
       <c r="C91" s="5" t="n"/>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
-        <is>
-          <t>O QUE ESTA FICHA NÃO CALCULA, E POR QUÊ</t>
-        </is>
-      </c>
-      <c r="AK91" s="5" t="n"/>
-      <c r="AL91" s="5" t="n"/>
-      <c r="AM91" s="5" t="n"/>
-      <c r="AN91" s="5" t="n"/>
-      <c r="AO91" s="5" t="n"/>
-      <c r="AP91" s="5" t="n"/>
-      <c r="AQ91" s="5" t="n"/>
-      <c r="AR91" s="5" t="n"/>
-      <c r="AS91" s="5" t="n"/>
-      <c r="AT91" s="5" t="n"/>
+      <c r="D91" s="35" t="inlineStr">
+        <is>
+          <t>comandar</t>
+        </is>
+      </c>
+      <c r="M91" s="36">
+        <f>"a Ação Padrão, toda rodada"</f>
+        <v/>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="1" t="n"/>
       <c r="B92" s="1" t="n"/>
       <c r="C92" s="5" t="n"/>
-      <c r="G92" s="5" t="n"/>
-      <c r="H92" s="5" t="n"/>
-      <c r="I92" s="5" t="n"/>
-      <c r="J92" s="5" t="n"/>
-      <c r="K92" s="5" t="n"/>
-      <c r="L92" s="5" t="n"/>
-      <c r="M92" s="5" t="n"/>
-      <c r="N92" s="5" t="n"/>
-      <c r="O92" s="5" t="n"/>
-      <c r="P92" s="5" t="n"/>
-      <c r="Q92" s="5" t="n"/>
-      <c r="R92" s="5" t="n"/>
-      <c r="S92" s="5" t="n"/>
-      <c r="T92" s="5" t="n"/>
-      <c r="U92" s="5" t="n"/>
-      <c r="V92" s="5" t="n"/>
-      <c r="W92" s="5" t="n"/>
-      <c r="X92" s="5" t="n"/>
-      <c r="Y92" s="5" t="n"/>
-      <c r="Z92" s="5" t="n"/>
-      <c r="AA92" s="5" t="n"/>
-      <c r="AB92" s="5" t="n"/>
-      <c r="AC92" s="5" t="n"/>
-      <c r="AD92" s="5" t="n"/>
-      <c r="AE92" s="5" t="n"/>
-      <c r="AF92" s="5" t="n"/>
-      <c r="AG92" s="5" t="n"/>
-      <c r="AH92" s="5" t="n"/>
-      <c r="AI92" s="5" t="n"/>
-      <c r="AJ92" s="5" t="n"/>
-      <c r="AK92" s="5" t="n"/>
-      <c r="AL92" s="5" t="n"/>
-      <c r="AM92" s="5" t="n"/>
-      <c r="AN92" s="5" t="n"/>
-      <c r="AO92" s="5" t="n"/>
-      <c r="AP92" s="5" t="n"/>
-      <c r="AQ92" s="5" t="n"/>
-      <c r="AR92" s="5" t="n"/>
-      <c r="AS92" s="5" t="n"/>
-      <c r="AT92" s="5" t="n"/>
+      <c r="D92" s="33" t="inlineStr">
+        <is>
+          <t>iniciativa</t>
+        </is>
+      </c>
+      <c r="M92" s="34">
+        <f>"a sua, e ela age logo depois de você"</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
-      <c r="D93" s="37" t="inlineStr">
+      <c r="D93" s="35" t="inlineStr">
+        <is>
+          <t>deslocamento</t>
+        </is>
+      </c>
+      <c r="M93" s="36">
+        <f>(9&amp;" metros")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="D94" s="33" t="inlineStr">
+        <is>
+          <t>amarra</t>
+        </is>
+      </c>
+      <c r="M94" s="34">
+        <f>(18&amp;" metros — além disso não pode ser comandada, e não some")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="D96" s="37" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="G96" s="38" t="inlineStr">
+        <is>
+          <t>O QUE ESTA FICHA NÃO CALCULA, E POR QUÊ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97"/>
+    <row r="98">
+      <c r="D98" s="39" t="inlineStr">
         <is>
           <t>a CD dos efeitos dela</t>
         </is>
       </c>
-      <c r="U93" s="38" t="n"/>
-      <c r="V93" s="38" t="n"/>
-      <c r="W93" s="38" t="n"/>
-      <c r="X93" s="38" t="n"/>
-      <c r="Y93" s="38" t="n"/>
-      <c r="Z93" s="38" t="n"/>
-      <c r="AA93" s="38" t="n"/>
-      <c r="AB93" s="38" t="n"/>
-      <c r="AC93" s="38" t="n"/>
-      <c r="AD93" s="38" t="n"/>
-      <c r="AE93" s="38" t="n"/>
-      <c r="AF93" s="38" t="n"/>
-      <c r="AG93" s="38" t="n"/>
-      <c r="AH93" s="38" t="n"/>
-      <c r="AI93" s="38" t="n"/>
-      <c r="AJ93" s="38" t="n"/>
-      <c r="AK93" s="38" t="n"/>
-      <c r="AL93" s="38" t="n"/>
-      <c r="AM93" s="38" t="n"/>
-      <c r="AN93" s="38" t="n"/>
-      <c r="AO93" s="38" t="n"/>
-      <c r="AP93" s="38" t="n"/>
-      <c r="AQ93" s="38" t="n"/>
-      <c r="AR93" s="38" t="n"/>
-      <c r="AS93" s="38" t="n"/>
-      <c r="AT93" s="38" t="n"/>
-    </row>
-    <row r="94">
-      <c r="D94" s="39">
+      <c r="U98" s="40" t="n"/>
+      <c r="V98" s="40" t="n"/>
+      <c r="W98" s="40" t="n"/>
+      <c r="X98" s="40" t="n"/>
+      <c r="Y98" s="40" t="n"/>
+      <c r="Z98" s="40" t="n"/>
+      <c r="AA98" s="40" t="n"/>
+      <c r="AB98" s="40" t="n"/>
+      <c r="AC98" s="40" t="n"/>
+      <c r="AD98" s="40" t="n"/>
+      <c r="AE98" s="40" t="n"/>
+      <c r="AF98" s="40" t="n"/>
+      <c r="AG98" s="40" t="n"/>
+      <c r="AH98" s="40" t="n"/>
+      <c r="AI98" s="40" t="n"/>
+      <c r="AJ98" s="40" t="n"/>
+      <c r="AK98" s="40" t="n"/>
+      <c r="AL98" s="40" t="n"/>
+      <c r="AM98" s="40" t="n"/>
+      <c r="AN98" s="40" t="n"/>
+      <c r="AO98" s="40" t="n"/>
+      <c r="AP98" s="40" t="n"/>
+      <c r="AQ98" s="40" t="n"/>
+      <c r="AR98" s="40" t="n"/>
+      <c r="AS98" s="40" t="n"/>
+      <c r="AT98" s="40" t="n"/>
+    </row>
+    <row r="99">
+      <c r="D99" s="41">
         <f>IF($AI$14="Voz","a Voz manda subir a CD dela, e a invocação não tem fórmula de CD em documento nenhum — combine com o mestre","")</f>
         <v/>
       </c>
     </row>
-    <row r="95">
-      <c r="D95" s="40" t="inlineStr">
+    <row r="100">
+      <c r="D100" s="42" t="inlineStr">
         <is>
           <t>A invocação não tem fórmula de CD em documento nenhum — nem o capítulo 16, nem a peça 15 escrevem uma. Esta rota soma num número que o sistema ainda não produz, então combine com o mestre em vez de chutar.</t>
         </is>
       </c>
     </row>
-    <row r="96"/>
+    <row r="101"/>
   </sheetData>
-  <mergeCells count="148">
+  <mergeCells count="162">
     <mergeCell ref="AI39:AM39"/>
-    <mergeCell ref="D86:L86"/>
     <mergeCell ref="D58:F59"/>
     <mergeCell ref="AI13:AS13"/>
     <mergeCell ref="D19:F20"/>
     <mergeCell ref="Q68:U68"/>
-    <mergeCell ref="M85:AT85"/>
     <mergeCell ref="D68:P68"/>
     <mergeCell ref="AN47:AS47"/>
     <mergeCell ref="M52:T52"/>
@@ -3777,142 +3847,158 @@
     <mergeCell ref="AM33:AS33"/>
     <mergeCell ref="D67:P67"/>
     <mergeCell ref="Y6:AD6"/>
+    <mergeCell ref="Q72:U72"/>
     <mergeCell ref="D1:AD2"/>
-    <mergeCell ref="T70:AT70"/>
+    <mergeCell ref="D69:P69"/>
     <mergeCell ref="A8:B26"/>
     <mergeCell ref="K7:P7"/>
     <mergeCell ref="G4:AD4"/>
-    <mergeCell ref="M87:AT87"/>
     <mergeCell ref="D33:L33"/>
     <mergeCell ref="D64:U64"/>
     <mergeCell ref="D45:F46"/>
     <mergeCell ref="Z66:AL66"/>
-    <mergeCell ref="D88:L88"/>
     <mergeCell ref="D26:L26"/>
     <mergeCell ref="N26:V26"/>
+    <mergeCell ref="D76:J76"/>
     <mergeCell ref="Q65:U65"/>
-    <mergeCell ref="D93:T93"/>
-    <mergeCell ref="T71:AT72"/>
-    <mergeCell ref="M88:AT88"/>
+    <mergeCell ref="Q70:U70"/>
     <mergeCell ref="AM65:AQ65"/>
+    <mergeCell ref="D70:P70"/>
+    <mergeCell ref="D83:K83"/>
+    <mergeCell ref="D90:L90"/>
     <mergeCell ref="N25:V25"/>
+    <mergeCell ref="D75:J75"/>
     <mergeCell ref="D47:J47"/>
+    <mergeCell ref="D86:AT86"/>
     <mergeCell ref="D6:I6"/>
     <mergeCell ref="Q66:U66"/>
     <mergeCell ref="D36:L36"/>
+    <mergeCell ref="D72:P72"/>
     <mergeCell ref="AF22:AK23"/>
     <mergeCell ref="D21:I21"/>
     <mergeCell ref="N36:U36"/>
+    <mergeCell ref="L76:R76"/>
+    <mergeCell ref="M90:AT90"/>
     <mergeCell ref="R6:W6"/>
+    <mergeCell ref="D71:P71"/>
     <mergeCell ref="AM7:AS7"/>
+    <mergeCell ref="D84:K84"/>
     <mergeCell ref="V52:AC52"/>
     <mergeCell ref="R21:W21"/>
     <mergeCell ref="D7:I7"/>
+    <mergeCell ref="D73:P73"/>
     <mergeCell ref="O39:S39"/>
     <mergeCell ref="N37:U37"/>
+    <mergeCell ref="M91:AT91"/>
     <mergeCell ref="D37:L37"/>
-    <mergeCell ref="G83:AD83"/>
-    <mergeCell ref="L70:R70"/>
     <mergeCell ref="Q67:U67"/>
     <mergeCell ref="L48:R48"/>
     <mergeCell ref="Z65:AL65"/>
     <mergeCell ref="AF32:AK32"/>
     <mergeCell ref="AM67:AQ67"/>
+    <mergeCell ref="M93:AT93"/>
     <mergeCell ref="AE51:AT51"/>
     <mergeCell ref="G45:AD45"/>
+    <mergeCell ref="D79:AT79"/>
     <mergeCell ref="D11:F12"/>
-    <mergeCell ref="D95:AT96"/>
+    <mergeCell ref="T75:AT75"/>
+    <mergeCell ref="Q69:U69"/>
     <mergeCell ref="AF7:AK7"/>
     <mergeCell ref="D35:AT35"/>
     <mergeCell ref="L47:R47"/>
-    <mergeCell ref="D78:K78"/>
-    <mergeCell ref="D89:L89"/>
+    <mergeCell ref="M92:AT92"/>
+    <mergeCell ref="AM69:AQ69"/>
     <mergeCell ref="V51:AC51"/>
     <mergeCell ref="D14:O14"/>
-    <mergeCell ref="D81:AT81"/>
+    <mergeCell ref="D99:AT99"/>
     <mergeCell ref="T48:AE48"/>
-    <mergeCell ref="N78:X78"/>
     <mergeCell ref="AF33:AK33"/>
     <mergeCell ref="G19:AH19"/>
     <mergeCell ref="D51:K51"/>
     <mergeCell ref="K21:P21"/>
     <mergeCell ref="R22:W23"/>
+    <mergeCell ref="T76:AT77"/>
     <mergeCell ref="Y21:AD21"/>
     <mergeCell ref="Z67:AL67"/>
     <mergeCell ref="Q14:Y14"/>
     <mergeCell ref="X39:AH39"/>
     <mergeCell ref="D30:F31"/>
+    <mergeCell ref="D100:AT101"/>
+    <mergeCell ref="Q71:U71"/>
+    <mergeCell ref="D88:F89"/>
     <mergeCell ref="D28:AT28"/>
+    <mergeCell ref="Z69:AL69"/>
+    <mergeCell ref="G81:AF81"/>
+    <mergeCell ref="D91:L91"/>
     <mergeCell ref="AM66:AQ66"/>
     <mergeCell ref="Y7:AD7"/>
     <mergeCell ref="AA14:AG14"/>
     <mergeCell ref="D9:AT9"/>
+    <mergeCell ref="D81:F82"/>
+    <mergeCell ref="Q73:U73"/>
     <mergeCell ref="M51:T51"/>
     <mergeCell ref="AM32:AS32"/>
+    <mergeCell ref="D93:L93"/>
     <mergeCell ref="G30:AJ30"/>
     <mergeCell ref="AM68:AQ68"/>
     <mergeCell ref="D25:L25"/>
-    <mergeCell ref="D94:AT94"/>
     <mergeCell ref="AN48:AS48"/>
+    <mergeCell ref="D92:L92"/>
     <mergeCell ref="X26:AR26"/>
-    <mergeCell ref="D76:F77"/>
     <mergeCell ref="D65:P65"/>
     <mergeCell ref="K6:P6"/>
-    <mergeCell ref="D85:L85"/>
     <mergeCell ref="D16:AT17"/>
     <mergeCell ref="X25:AR25"/>
     <mergeCell ref="K22:P23"/>
+    <mergeCell ref="D94:L94"/>
     <mergeCell ref="Y22:AD23"/>
-    <mergeCell ref="L71:R71"/>
+    <mergeCell ref="N84:AD84"/>
     <mergeCell ref="N32:S32"/>
     <mergeCell ref="D39:N39"/>
+    <mergeCell ref="G96:AJ96"/>
+    <mergeCell ref="M94:AT94"/>
     <mergeCell ref="D66:P66"/>
+    <mergeCell ref="D98:T98"/>
     <mergeCell ref="A30:B48"/>
     <mergeCell ref="Z68:AL68"/>
-    <mergeCell ref="D79:K79"/>
     <mergeCell ref="R7:W7"/>
-    <mergeCell ref="D71:J71"/>
     <mergeCell ref="U33:AD33"/>
-    <mergeCell ref="N79:AD79"/>
     <mergeCell ref="D13:O13"/>
     <mergeCell ref="N33:S33"/>
-    <mergeCell ref="M86:AT86"/>
     <mergeCell ref="D32:L32"/>
     <mergeCell ref="D43:AT43"/>
     <mergeCell ref="AF6:AK6"/>
-    <mergeCell ref="M89:AT89"/>
     <mergeCell ref="AM6:AS6"/>
     <mergeCell ref="AG48:AL48"/>
     <mergeCell ref="AE52:AT53"/>
-    <mergeCell ref="D87:L87"/>
     <mergeCell ref="D52:K52"/>
-    <mergeCell ref="D74:AT74"/>
     <mergeCell ref="Z64:AQ64"/>
     <mergeCell ref="D22:I23"/>
     <mergeCell ref="AG47:AL47"/>
     <mergeCell ref="D60:J60"/>
+    <mergeCell ref="D96:F97"/>
     <mergeCell ref="G58:AJ58"/>
     <mergeCell ref="O41:S41"/>
     <mergeCell ref="D41:N41"/>
     <mergeCell ref="AI41:AM41"/>
     <mergeCell ref="AA13:AG13"/>
-    <mergeCell ref="G91:AJ91"/>
+    <mergeCell ref="G88:AD88"/>
+    <mergeCell ref="AM70:AQ70"/>
+    <mergeCell ref="L75:R75"/>
+    <mergeCell ref="Z70:AL70"/>
     <mergeCell ref="D4:F5"/>
     <mergeCell ref="Q13:Y13"/>
-    <mergeCell ref="D91:F92"/>
     <mergeCell ref="X41:AH41"/>
     <mergeCell ref="D61:J61"/>
     <mergeCell ref="U32:AD32"/>
-    <mergeCell ref="D70:J70"/>
     <mergeCell ref="D48:J48"/>
-    <mergeCell ref="D83:F84"/>
     <mergeCell ref="D55:AT56"/>
     <mergeCell ref="G11:AD11"/>
     <mergeCell ref="AF1:AT2"/>
     <mergeCell ref="AI14:AS14"/>
-    <mergeCell ref="G76:AF76"/>
+    <mergeCell ref="N83:X83"/>
   </mergeCells>
-  <dataValidations count="15">
+  <dataValidations count="22">
     <dataValidation sqref="Q14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DADOS!$A$2:$A$5</formula1>
     </dataValidation>
@@ -3946,6 +4032,21 @@
     <dataValidation sqref="D68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DADOS!$H$2:$H$15</formula1>
     </dataValidation>
+    <dataValidation sqref="D69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$H$2:$H$15</formula1>
+    </dataValidation>
+    <dataValidation sqref="D70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$H$2:$H$15</formula1>
+    </dataValidation>
+    <dataValidation sqref="D71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$H$2:$H$15</formula1>
+    </dataValidation>
+    <dataValidation sqref="D72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$H$2:$H$15</formula1>
+    </dataValidation>
+    <dataValidation sqref="D73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$H$2:$H$15</formula1>
+    </dataValidation>
     <dataValidation sqref="Z65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DADOS!$I$2:$I$9</formula1>
     </dataValidation>
@@ -3956,6 +4057,12 @@
       <formula1>DADOS!$I$2:$I$9</formula1>
     </dataValidation>
     <dataValidation sqref="Z68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$I$2:$I$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DADOS!$I$2:$I$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DADOS!$I$2:$I$9</formula1>
     </dataValidation>
   </dataValidations>
@@ -3970,7 +4077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN55"/>
+  <dimension ref="A1:AN69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4007,60 +4114,60 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="41" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>tipos</t>
         </is>
       </c>
-      <c r="B1" s="41" t="inlineStr">
+      <c r="B1" s="43" t="inlineStr">
         <is>
           <t>trilhas</t>
         </is>
       </c>
-      <c r="C1" s="41" t="inlineStr">
+      <c r="C1" s="43" t="inlineStr">
         <is>
           <t>atributos</t>
         </is>
       </c>
-      <c r="D1" s="41" t="inlineStr">
+      <c r="D1" s="43" t="inlineStr">
         <is>
           <t>trs</t>
         </is>
       </c>
-      <c r="E1" s="41" t="inlineStr">
+      <c r="E1" s="43" t="inlineStr">
         <is>
           <t>sintonia</t>
         </is>
       </c>
-      <c r="F1" s="41" t="inlineStr">
+      <c r="F1" s="43" t="inlineStr">
         <is>
           <t>defesa_de</t>
         </is>
       </c>
-      <c r="G1" s="41" t="inlineStr">
+      <c r="G1" s="43" t="inlineStr">
         <is>
           <t>fisico_de</t>
         </is>
       </c>
-      <c r="H1" s="41" t="inlineStr">
+      <c r="H1" s="43" t="inlineStr">
         <is>
           <t>traco</t>
         </is>
       </c>
-      <c r="I1" s="41" t="inlineStr">
+      <c r="I1" s="43" t="inlineStr">
         <is>
           <t>comando</t>
         </is>
       </c>
       <c r="J1" s="5" t="n"/>
-      <c r="K1" s="41" t="inlineStr">
+      <c r="K1" s="43" t="inlineStr">
         <is>
           <t>tab_tipos</t>
         </is>
       </c>
       <c r="L1" s="5" t="n"/>
       <c r="M1" s="5" t="n"/>
-      <c r="N1" s="41" t="inlineStr">
+      <c r="N1" s="43" t="inlineStr">
         <is>
           <t>tab_trilhas</t>
         </is>
@@ -4070,21 +4177,21 @@
       <c r="Q1" s="5" t="n"/>
       <c r="R1" s="5" t="n"/>
       <c r="S1" s="5" t="n"/>
-      <c r="T1" s="41" t="inlineStr">
+      <c r="T1" s="43" t="inlineStr">
         <is>
           <t>tab_traco</t>
         </is>
       </c>
       <c r="U1" s="5" t="n"/>
       <c r="V1" s="5" t="n"/>
-      <c r="W1" s="41" t="inlineStr">
+      <c r="W1" s="43" t="inlineStr">
         <is>
           <t>tab_comando</t>
         </is>
       </c>
       <c r="X1" s="5" t="n"/>
       <c r="Y1" s="5" t="n"/>
-      <c r="Z1" s="41" t="inlineStr">
+      <c r="Z1" s="43" t="inlineStr">
         <is>
           <t>tab_investir</t>
         </is>
@@ -4092,7 +4199,7 @@
       <c r="AA1" s="5" t="n"/>
       <c r="AB1" s="5" t="n"/>
       <c r="AC1" s="5" t="n"/>
-      <c r="AD1" s="41" t="inlineStr">
+      <c r="AD1" s="43" t="inlineStr">
         <is>
           <t>tab_trs</t>
         </is>
@@ -4154,120 +4261,120 @@
         </is>
       </c>
       <c r="J2" s="5" t="n"/>
-      <c r="K2" s="42" t="inlineStr">
+      <c r="K2" s="44" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="L2" s="42" t="inlineStr">
+      <c r="L2" s="44" t="inlineStr">
         <is>
           <t>base</t>
         </is>
       </c>
       <c r="M2" s="5" t="n"/>
-      <c r="N2" s="42" t="inlineStr">
+      <c r="N2" s="44" t="inlineStr">
         <is>
           <t>trilha</t>
         </is>
       </c>
-      <c r="O2" s="42" t="inlineStr">
+      <c r="O2" s="44" t="inlineStr">
         <is>
           <t>corpos</t>
         </is>
       </c>
-      <c r="P2" s="42" t="inlineStr">
+      <c r="P2" s="44" t="inlineStr">
         <is>
           <t>mult</t>
         </is>
       </c>
-      <c r="Q2" s="42" t="inlineStr">
+      <c r="Q2" s="44" t="inlineStr">
         <is>
           <t>corpo</t>
         </is>
       </c>
-      <c r="R2" s="42" t="inlineStr">
+      <c r="R2" s="44" t="inlineStr">
         <is>
           <t>area</t>
         </is>
       </c>
       <c r="S2" s="5" t="n"/>
-      <c r="T2" s="42" t="inlineStr">
+      <c r="T2" s="44" t="inlineStr">
         <is>
           <t>traço</t>
         </is>
       </c>
-      <c r="U2" s="42" t="inlineStr">
+      <c r="U2" s="44" t="inlineStr">
         <is>
           <t>pontos</t>
         </is>
       </c>
       <c r="V2" s="5" t="n"/>
-      <c r="W2" s="42" t="inlineStr">
+      <c r="W2" s="44" t="inlineStr">
         <is>
           <t>comando</t>
         </is>
       </c>
-      <c r="X2" s="42" t="inlineStr">
+      <c r="X2" s="44" t="inlineStr">
         <is>
           <t>pontos</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n"/>
-      <c r="Z2" s="42" t="inlineStr">
+      <c r="Z2" s="44" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="AA2" s="42" t="inlineStr">
+      <c r="AA2" s="44" t="inlineStr">
         <is>
           <t>uma</t>
         </is>
       </c>
-      <c r="AB2" s="42" t="inlineStr">
+      <c r="AB2" s="44" t="inlineStr">
         <is>
           <t>matilha</t>
         </is>
       </c>
       <c r="AC2" s="5" t="n"/>
-      <c r="AD2" s="42" t="inlineStr">
+      <c r="AD2" s="44" t="inlineStr">
         <is>
           <t>tr</t>
         </is>
       </c>
-      <c r="AE2" s="42" t="inlineStr">
+      <c r="AE2" s="44" t="inlineStr">
         <is>
           <t>atributo</t>
         </is>
       </c>
       <c r="AF2" s="5" t="n"/>
-      <c r="AG2" s="42" t="inlineStr">
+      <c r="AG2" s="44" t="inlineStr">
         <is>
           <t>e_marcos</t>
         </is>
       </c>
-      <c r="AH2" s="42" t="inlineStr">
+      <c r="AH2" s="44" t="inlineStr">
         <is>
           <t>e_maestria</t>
         </is>
       </c>
-      <c r="AI2" s="42" t="inlineStr">
+      <c r="AI2" s="44" t="inlineStr">
         <is>
           <t>e_classe</t>
         </is>
       </c>
       <c r="AJ2" s="5" t="n"/>
-      <c r="AK2" s="42" t="inlineStr">
+      <c r="AK2" s="44" t="inlineStr">
         <is>
           <t>espelho</t>
         </is>
       </c>
       <c r="AL2" s="5" t="n"/>
-      <c r="AM2" s="42" t="inlineStr">
+      <c r="AM2" s="44" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="AN2" s="43" t="inlineStr">
+      <c r="AN2" s="45" t="inlineStr">
         <is>
           <t>célula</t>
         </is>
@@ -4412,7 +4519,7 @@
           <t>nivel</t>
         </is>
       </c>
-      <c r="AN3" s="44" t="inlineStr">
+      <c r="AN3" s="46" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
@@ -4549,7 +4656,7 @@
           <t>ess_dono</t>
         </is>
       </c>
-      <c r="AN4" s="44" t="inlineStr">
+      <c r="AN4" s="46" t="inlineStr">
         <is>
           <t>K7</t>
         </is>
@@ -4682,7 +4789,7 @@
           <t>int_dono</t>
         </is>
       </c>
-      <c r="AN5" s="44" t="inlineStr">
+      <c r="AN5" s="46" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
@@ -4787,7 +4894,7 @@
           <t>maestria</t>
         </is>
       </c>
-      <c r="AN6" s="44" t="inlineStr">
+      <c r="AN6" s="46" t="inlineStr">
         <is>
           <t>Y7</t>
         </is>
@@ -4874,7 +4981,7 @@
           <t>marcos</t>
         </is>
       </c>
-      <c r="AN7" s="44" t="inlineStr">
+      <c r="AN7" s="46" t="inlineStr">
         <is>
           <t>AF7</t>
         </is>
@@ -4958,7 +5065,7 @@
           <t>classe</t>
         </is>
       </c>
-      <c r="AN8" s="44" t="inlineStr">
+      <c r="AN8" s="46" t="inlineStr">
         <is>
           <t>AM7</t>
         </is>
@@ -5042,7 +5149,7 @@
           <t>nome</t>
         </is>
       </c>
-      <c r="AN9" s="44" t="inlineStr">
+      <c r="AN9" s="46" t="inlineStr">
         <is>
           <t>D14</t>
         </is>
@@ -5108,7 +5215,7 @@
           <t>tipo</t>
         </is>
       </c>
-      <c r="AN10" s="44" t="inlineStr">
+      <c r="AN10" s="46" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
@@ -5168,7 +5275,7 @@
           <t>trilha</t>
         </is>
       </c>
-      <c r="AN11" s="44" t="inlineStr">
+      <c r="AN11" s="46" t="inlineStr">
         <is>
           <t>AA14</t>
         </is>
@@ -5228,7 +5335,7 @@
           <t>sintonia</t>
         </is>
       </c>
-      <c r="AN12" s="44" t="inlineStr">
+      <c r="AN12" s="46" t="inlineStr">
         <is>
           <t>AI14</t>
         </is>
@@ -5288,7 +5395,7 @@
           <t>pontos_atributo</t>
         </is>
       </c>
-      <c r="AN13" s="44" t="inlineStr">
+      <c r="AN13" s="46" t="inlineStr">
         <is>
           <t>D26</t>
         </is>
@@ -5348,7 +5455,7 @@
           <t>pontos_disp</t>
         </is>
       </c>
-      <c r="AN14" s="44" t="inlineStr">
+      <c r="AN14" s="46" t="inlineStr">
         <is>
           <t>N26</t>
         </is>
@@ -5408,7 +5515,7 @@
           <t>aviso_atributo</t>
         </is>
       </c>
-      <c r="AN15" s="44" t="inlineStr">
+      <c r="AN15" s="46" t="inlineStr">
         <is>
           <t>X26</t>
         </is>
@@ -5464,7 +5571,7 @@
           <t>atr_acerto</t>
         </is>
       </c>
-      <c r="AN16" s="44" t="inlineStr">
+      <c r="AN16" s="46" t="inlineStr">
         <is>
           <t>D33</t>
         </is>
@@ -5514,7 +5621,7 @@
           <t>acerto</t>
         </is>
       </c>
-      <c r="AN17" s="44" t="inlineStr">
+      <c r="AN17" s="46" t="inlineStr">
         <is>
           <t>N33</t>
         </is>
@@ -5564,7 +5671,7 @@
           <t>defesa_de</t>
         </is>
       </c>
-      <c r="AN18" s="44" t="inlineStr">
+      <c r="AN18" s="46" t="inlineStr">
         <is>
           <t>U33</t>
         </is>
@@ -5614,7 +5721,7 @@
           <t>defesa</t>
         </is>
       </c>
-      <c r="AN19" s="44" t="inlineStr">
+      <c r="AN19" s="46" t="inlineStr">
         <is>
           <t>AF33</t>
         </is>
@@ -5664,7 +5771,7 @@
           <t>critico</t>
         </is>
       </c>
-      <c r="AN20" s="44" t="inlineStr">
+      <c r="AN20" s="46" t="inlineStr">
         <is>
           <t>AM33</t>
         </is>
@@ -5714,7 +5821,7 @@
           <t>tr_treinado</t>
         </is>
       </c>
-      <c r="AN21" s="44" t="inlineStr">
+      <c r="AN21" s="46" t="inlineStr">
         <is>
           <t>D37</t>
         </is>
@@ -5764,7 +5871,7 @@
           <t>fisico_de</t>
         </is>
       </c>
-      <c r="AN22" s="44" t="inlineStr">
+      <c r="AN22" s="46" t="inlineStr">
         <is>
           <t>N37</t>
         </is>
@@ -5814,7 +5921,7 @@
           <t>vida_max</t>
         </is>
       </c>
-      <c r="AN23" s="44" t="inlineStr">
+      <c r="AN23" s="46" t="inlineStr">
         <is>
           <t>D48</t>
         </is>
@@ -5864,7 +5971,7 @@
           <t>vida</t>
         </is>
       </c>
-      <c r="AN24" s="44" t="inlineStr">
+      <c r="AN24" s="46" t="inlineStr">
         <is>
           <t>L48</t>
         </is>
@@ -5914,7 +6021,7 @@
           <t>corpos</t>
         </is>
       </c>
-      <c r="AN25" s="44" t="inlineStr">
+      <c r="AN25" s="46" t="inlineStr">
         <is>
           <t>AG48</t>
         </is>
@@ -5964,7 +6071,7 @@
           <t>area</t>
         </is>
       </c>
-      <c r="AN26" s="44" t="inlineStr">
+      <c r="AN26" s="46" t="inlineStr">
         <is>
           <t>AN48</t>
         </is>
@@ -6014,7 +6121,7 @@
           <t>regua</t>
         </is>
       </c>
-      <c r="AN27" s="44" t="inlineStr">
+      <c r="AN27" s="46" t="inlineStr">
         <is>
           <t>D52</t>
         </is>
@@ -6064,7 +6171,7 @@
           <t>meia_regua</t>
         </is>
       </c>
-      <c r="AN28" s="44" t="inlineStr">
+      <c r="AN28" s="46" t="inlineStr">
         <is>
           <t>M52</t>
         </is>
@@ -6114,7 +6221,7 @@
           <t>volta_com</t>
         </is>
       </c>
-      <c r="AN29" s="44" t="inlineStr">
+      <c r="AN29" s="46" t="inlineStr">
         <is>
           <t>V52</t>
         </is>
@@ -6164,309 +6271,477 @@
           <t>orcamento</t>
         </is>
       </c>
-      <c r="AN30" s="44" t="inlineStr">
+      <c r="AN30" s="46" t="inlineStr">
         <is>
           <t>D61</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="AM31" s="44" t="inlineStr">
+      <c r="AM31" s="46" t="inlineStr">
         <is>
           <t>gasto</t>
         </is>
       </c>
-      <c r="AN31" s="44" t="inlineStr">
+      <c r="AN31" s="46" t="inlineStr">
+        <is>
+          <t>D76</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="AM32" s="46" t="inlineStr">
+        <is>
+          <t>sobra</t>
+        </is>
+      </c>
+      <c r="AN32" s="46" t="inlineStr">
+        <is>
+          <t>L76</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="AM33" s="46" t="inlineStr">
+        <is>
+          <t>investir</t>
+        </is>
+      </c>
+      <c r="AN33" s="46" t="inlineStr">
+        <is>
+          <t>D84</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="AM34" s="46" t="inlineStr">
+        <is>
+          <t>cd_pendente</t>
+        </is>
+      </c>
+      <c r="AN34" s="46" t="inlineStr">
+        <is>
+          <t>D99</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="AM35" s="46" t="inlineStr">
+        <is>
+          <t>atr_Força</t>
+        </is>
+      </c>
+      <c r="AN35" s="46" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="AM36" s="46" t="inlineStr">
+        <is>
+          <t>atr_Destreza</t>
+        </is>
+      </c>
+      <c r="AN36" s="46" t="inlineStr">
+        <is>
+          <t>K22</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="AM37" s="46" t="inlineStr">
+        <is>
+          <t>atr_Constituição</t>
+        </is>
+      </c>
+      <c r="AN37" s="46" t="inlineStr">
+        <is>
+          <t>R22</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="AM38" s="46" t="inlineStr">
+        <is>
+          <t>atr_Inteligência</t>
+        </is>
+      </c>
+      <c r="AN38" s="46" t="inlineStr">
+        <is>
+          <t>Y22</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="AM39" s="46" t="inlineStr">
+        <is>
+          <t>atr_Essência</t>
+        </is>
+      </c>
+      <c r="AN39" s="46" t="inlineStr">
+        <is>
+          <t>AF22</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="AM40" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_1</t>
+        </is>
+      </c>
+      <c r="AN40" s="46" t="inlineStr">
+        <is>
+          <t>Q65</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="AM41" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_2</t>
+        </is>
+      </c>
+      <c r="AN41" s="46" t="inlineStr">
+        <is>
+          <t>Q66</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="AM42" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_3</t>
+        </is>
+      </c>
+      <c r="AN42" s="46" t="inlineStr">
+        <is>
+          <t>Q67</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="AM43" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_4</t>
+        </is>
+      </c>
+      <c r="AN43" s="46" t="inlineStr">
+        <is>
+          <t>Q68</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="AM44" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_5</t>
+        </is>
+      </c>
+      <c r="AN44" s="46" t="inlineStr">
+        <is>
+          <t>Q69</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="AM45" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_6</t>
+        </is>
+      </c>
+      <c r="AN45" s="46" t="inlineStr">
+        <is>
+          <t>Q70</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="AM46" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_7</t>
+        </is>
+      </c>
+      <c r="AN46" s="46" t="inlineStr">
+        <is>
+          <t>Q71</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="AM47" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_8</t>
+        </is>
+      </c>
+      <c r="AN47" s="46" t="inlineStr">
+        <is>
+          <t>Q72</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="AM48" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_9</t>
+        </is>
+      </c>
+      <c r="AN48" s="46" t="inlineStr">
+        <is>
+          <t>Q73</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="AM49" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_10</t>
+        </is>
+      </c>
+      <c r="AN49" s="46" t="inlineStr">
+        <is>
+          <t>AM65</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="AM50" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_11</t>
+        </is>
+      </c>
+      <c r="AN50" s="46" t="inlineStr">
+        <is>
+          <t>AM66</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="AM51" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_12</t>
+        </is>
+      </c>
+      <c r="AN51" s="46" t="inlineStr">
+        <is>
+          <t>AM67</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="AM52" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_13</t>
+        </is>
+      </c>
+      <c r="AN52" s="46" t="inlineStr">
+        <is>
+          <t>AM68</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="AM53" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_14</t>
+        </is>
+      </c>
+      <c r="AN53" s="46" t="inlineStr">
+        <is>
+          <t>AM69</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="AM54" s="46" t="inlineStr">
+        <is>
+          <t>slot_pontos_15</t>
+        </is>
+      </c>
+      <c r="AN54" s="46" t="inlineStr">
+        <is>
+          <t>AM70</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="AM55" s="46" t="inlineStr">
+        <is>
+          <t>traco_1</t>
+        </is>
+      </c>
+      <c r="AN55" s="46" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="AM56" s="46" t="inlineStr">
+        <is>
+          <t>traco_2</t>
+        </is>
+      </c>
+      <c r="AN56" s="46" t="inlineStr">
+        <is>
+          <t>D66</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="AM57" s="46" t="inlineStr">
+        <is>
+          <t>traco_3</t>
+        </is>
+      </c>
+      <c r="AN57" s="46" t="inlineStr">
+        <is>
+          <t>D67</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="AM58" s="46" t="inlineStr">
+        <is>
+          <t>traco_4</t>
+        </is>
+      </c>
+      <c r="AN58" s="46" t="inlineStr">
+        <is>
+          <t>D68</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="AM59" s="46" t="inlineStr">
+        <is>
+          <t>traco_5</t>
+        </is>
+      </c>
+      <c r="AN59" s="46" t="inlineStr">
+        <is>
+          <t>D69</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="AM60" s="46" t="inlineStr">
+        <is>
+          <t>traco_6</t>
+        </is>
+      </c>
+      <c r="AN60" s="46" t="inlineStr">
+        <is>
+          <t>D70</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="AM61" s="46" t="inlineStr">
+        <is>
+          <t>traco_7</t>
+        </is>
+      </c>
+      <c r="AN61" s="46" t="inlineStr">
         <is>
           <t>D71</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="AM32" s="44" t="inlineStr">
-        <is>
-          <t>sobra</t>
-        </is>
-      </c>
-      <c r="AN32" s="44" t="inlineStr">
-        <is>
-          <t>L71</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="AM33" s="44" t="inlineStr">
-        <is>
-          <t>investir</t>
-        </is>
-      </c>
-      <c r="AN33" s="44" t="inlineStr">
-        <is>
-          <t>D79</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="AM34" s="44" t="inlineStr">
-        <is>
-          <t>cd_pendente</t>
-        </is>
-      </c>
-      <c r="AN34" s="44" t="inlineStr">
-        <is>
-          <t>D94</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="AM35" s="44" t="inlineStr">
-        <is>
-          <t>atr_Força</t>
-        </is>
-      </c>
-      <c r="AN35" s="44" t="inlineStr">
-        <is>
-          <t>D22</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="AM36" s="44" t="inlineStr">
-        <is>
-          <t>atr_Destreza</t>
-        </is>
-      </c>
-      <c r="AN36" s="44" t="inlineStr">
-        <is>
-          <t>K22</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="AM37" s="44" t="inlineStr">
-        <is>
-          <t>atr_Constituição</t>
-        </is>
-      </c>
-      <c r="AN37" s="44" t="inlineStr">
-        <is>
-          <t>R22</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="AM38" s="44" t="inlineStr">
-        <is>
-          <t>atr_Inteligência</t>
-        </is>
-      </c>
-      <c r="AN38" s="44" t="inlineStr">
-        <is>
-          <t>Y22</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="AM39" s="44" t="inlineStr">
-        <is>
-          <t>atr_Essência</t>
-        </is>
-      </c>
-      <c r="AN39" s="44" t="inlineStr">
-        <is>
-          <t>AF22</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="AM40" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_1</t>
-        </is>
-      </c>
-      <c r="AN40" s="44" t="inlineStr">
-        <is>
-          <t>Q65</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="AM41" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_2</t>
-        </is>
-      </c>
-      <c r="AN41" s="44" t="inlineStr">
-        <is>
-          <t>Q66</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="AM42" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_3</t>
-        </is>
-      </c>
-      <c r="AN42" s="44" t="inlineStr">
-        <is>
-          <t>Q67</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="AM43" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_4</t>
-        </is>
-      </c>
-      <c r="AN43" s="44" t="inlineStr">
-        <is>
-          <t>Q68</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="AM44" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_5</t>
-        </is>
-      </c>
-      <c r="AN44" s="44" t="inlineStr">
-        <is>
-          <t>AM65</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="AM45" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_6</t>
-        </is>
-      </c>
-      <c r="AN45" s="44" t="inlineStr">
-        <is>
-          <t>AM66</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="AM46" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_7</t>
-        </is>
-      </c>
-      <c r="AN46" s="44" t="inlineStr">
-        <is>
-          <t>AM67</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="AM47" s="44" t="inlineStr">
-        <is>
-          <t>slot_pontos_8</t>
-        </is>
-      </c>
-      <c r="AN47" s="44" t="inlineStr">
-        <is>
-          <t>AM68</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="AM48" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_1</t>
-        </is>
-      </c>
-      <c r="AN48" s="44" t="inlineStr">
-        <is>
-          <t>D65</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="AM49" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_2</t>
-        </is>
-      </c>
-      <c r="AN49" s="44" t="inlineStr">
-        <is>
-          <t>D66</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="AM50" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_3</t>
-        </is>
-      </c>
-      <c r="AN50" s="44" t="inlineStr">
-        <is>
-          <t>D67</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="AM51" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_4</t>
-        </is>
-      </c>
-      <c r="AN51" s="44" t="inlineStr">
-        <is>
-          <t>D68</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="AM52" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_5</t>
-        </is>
-      </c>
-      <c r="AN52" s="44" t="inlineStr">
+    <row r="62">
+      <c r="AM62" s="46" t="inlineStr">
+        <is>
+          <t>traco_8</t>
+        </is>
+      </c>
+      <c r="AN62" s="46" t="inlineStr">
+        <is>
+          <t>D72</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="AM63" s="46" t="inlineStr">
+        <is>
+          <t>traco_9</t>
+        </is>
+      </c>
+      <c r="AN63" s="46" t="inlineStr">
+        <is>
+          <t>D73</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="AM64" s="46" t="inlineStr">
+        <is>
+          <t>comando_1</t>
+        </is>
+      </c>
+      <c r="AN64" s="46" t="inlineStr">
         <is>
           <t>Z65</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="AM53" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_6</t>
-        </is>
-      </c>
-      <c r="AN53" s="44" t="inlineStr">
+    <row r="65">
+      <c r="AM65" s="46" t="inlineStr">
+        <is>
+          <t>comando_2</t>
+        </is>
+      </c>
+      <c r="AN65" s="46" t="inlineStr">
         <is>
           <t>Z66</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="AM54" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_7</t>
-        </is>
-      </c>
-      <c r="AN54" s="44" t="inlineStr">
+    <row r="66">
+      <c r="AM66" s="46" t="inlineStr">
+        <is>
+          <t>comando_3</t>
+        </is>
+      </c>
+      <c r="AN66" s="46" t="inlineStr">
         <is>
           <t>Z67</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="AM55" s="44" t="inlineStr">
-        <is>
-          <t>slot_nome_8</t>
-        </is>
-      </c>
-      <c r="AN55" s="44" t="inlineStr">
+    <row r="67">
+      <c r="AM67" s="46" t="inlineStr">
+        <is>
+          <t>comando_4</t>
+        </is>
+      </c>
+      <c r="AN67" s="46" t="inlineStr">
         <is>
           <t>Z68</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="AM68" s="46" t="inlineStr">
+        <is>
+          <t>comando_5</t>
+        </is>
+      </c>
+      <c r="AN68" s="46" t="inlineStr">
+        <is>
+          <t>Z69</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="AM69" s="46" t="inlineStr">
+        <is>
+          <t>comando_6</t>
+        </is>
+      </c>
+      <c r="AN69" s="46" t="inlineStr">
+        <is>
+          <t>Z70</t>
         </is>
       </c>
     </row>

</xml_diff>